<commit_message>
Align host cities page keyword and URL
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -11,9 +11,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="72" customWidth="1"/>
+    <col min="4" max="4" width="82" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
@@ -212,7 +212,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>/world-cup-2026-host-cities/</t>
+          <t>/world-cup-2026-schedule-host-cities/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -222,7 +222,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Host city planner、搜索/国家/规划需求/排序、城市卡片、快捷预设、决策卡、banner</t>
+          <t>唯一核心关键词改为world-cup-2026-schedule-host-cities；URL、H1、Title、Meta、内链、旧URL跳转已同步</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>

<commit_message>
Optimize schedule host cities SEO content
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -13,7 +13,7 @@
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="82" customWidth="1"/>
+    <col min="4" max="4" width="88" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
@@ -217,12 +217,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>已完成阶段性优化</t>
+          <t>已完成SEO内容优化</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>唯一核心关键词改为world-cup-2026-schedule-host-cities；URL、H1、Title、Meta、内链、旧URL跳转已同步</t>
+          <t>唯一核心关键词、URL、H1已统一；新增官方来源模块、HowTo Schema、5个FAQ、页面专属使用表；关键词族密度4.92%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>

<commit_message>
Update schedule host cities title and description
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -12,8 +12,8 @@
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="88" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="96" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
@@ -217,12 +217,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>已完成SEO内容优化</t>
+          <t>已完成Title/Description重优化</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>唯一核心关键词、URL、H1已统一；新增官方来源模块、HowTo Schema、5个FAQ、页面专属使用表；关键词族密度4.92%</t>
+          <t>Title和Description已按用户指定文本精确输出；H2与来源模块同步强化full match dates、venues、fixtures、knockout rounds、semifinals、third-place match、final details</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>

<commit_message>
Improve host cities hero planner
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -14,7 +14,7 @@
     <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="96" customWidth="1"/>
-    <col min="5" max="5" width="48" customWidth="1"/>
+    <col min="5" max="5" width="52" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
@@ -217,12 +217,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>已完成Title/Description重优化</t>
+          <t>已完成首屏交互优化</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Title和Description已按用户指定文本精确输出；H2与来源模块同步强化full match dates、venues、fixtures、knockout rounds、semifinals、third-place match、final details</t>
+          <t>左侧首屏文案已按核心关键词SEO/GEO重写；右侧静态面板改为可筛选城市/规划需求的功能控制面板，可联动下方Host city planner并高亮结果</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>

<commit_message>
Add AdSense readiness checklist
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -426,6 +426,43 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AdSense 技术准备项</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>全站验证 / ads.txt / 合规页面 / 广告加载开关</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>已加入开发清单，待上线前配置</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>已明确预留 head 验证、/ads.txt、Privacy Policy、About、Contact、Disclaimer、移动端体验和正式申请前检查项</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>网站内容完成并部署到 worldcup2026schedule.net 后，使用正式 AdSense 账号信息完成验证</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add AdSense trust pages
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -463,6 +463,43 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AdSense 信任与合规页面</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>/privacy-policy/ /about/ /contact/ /disclaimer/</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>已创建4个合规基础页面；已加入footer入口和sitemap；每页包含独立说明、FAQ、canonical和Schema</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>上线前配置真实联系邮箱；拿到AdSense账号后再添加验证代码和ads.txt</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add AdSense verification infrastructure
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -500,6 +500,43 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AdSense 验证基础设施</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Head验证位 / AdSense脚本开关 / ads.txt / .env.example</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>已实现ADSENSE_PUBLISHER_ID、验证方式、脚本加载和ads.txt开关；默认构建不输出验证标签、不加载广告脚本、不写入假publisher ID</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>部署到worldcup2026schedule.net后，使用正式AdSense账号ID配置生产环境变量并验证源码</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve host city comparison filters
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -537,6 +537,43 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Host Cities Phase B</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-host-cities/</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>已新增Region筛选、4个交互式城市比较卡、16个城市价值标签、16个Planning highlight模块；关键词密度回到4.67%</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>下一步可优化单个高优先级城市详情页，或继续做Groups页面工具化</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add visual host city cards
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -574,6 +574,43 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Host Cities Phase C</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-host-cities/</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>已接入16张城市图片资源；新增8张视觉Featured City Cards，包含城市图、路线标签、球场、比赛数、容量和Open city guide入口</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>下一步可继续优化城市详情页，或为16个城市补充独立图片卡排序/横向滚动体验</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Show all host city visual cards
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1,616 +1,1058 @@
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="任务进度" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务进度" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="38" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="96" customWidth="1"/>
-    <col min="5" max="5" width="52" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="96" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>任务模块</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>页面/范围</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>当前状态</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>完成内容</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>下一步动作</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>负责人</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>更新时间</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>基础规划</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>网站开发方案 / 关键词方案 / 内容方案 / SEO方案</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>已生成本地指导文件，并用于后续页面优化</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>持续按页面复盘更新</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Schedule 页面</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-schedule/</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>已完成阶段性优化</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>完整赛程、导出、Team/City View、时区、动态比赛、Match Detail、控制面板、banner</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>后续做性能和结构化数据统一检查</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>PDF 页面</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-schedule-pdf/</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>已完成阶段性优化</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>PDF库、文件选择、主题hero、功能卡片、关键词补强、banner</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>后续检查下载文件命名和Schema</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Excel 页面</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-schedule-excel/</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>已完成阶段性优化</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Excel/CSV选择、Spreadsheet planner、主题hero、banner</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>后续检查文件字段说明和使用教程</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Host Cities 页面</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-schedule-host-cities/</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>已完成首屏交互优化</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>左侧首屏文案已按核心关键词SEO/GEO重写；右侧静态面板改为可筛选城市/规划需求的功能控制面板，可联动下方Host city planner并高亮结果</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>下一步可优化单个城市详情页或Groups页面</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Groups 页面</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-groups/</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>未开始</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>待按SEO方案做分组和晋级规划工具化</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>建议作为下一项页面优化</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Dates 页面</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-schedule-dates/</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>未开始</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>待升级为日期导航和比赛日规划页</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>排入下一阶段页面优化</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>TV 页面</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-tv-schedule/</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>未开始</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>待围绕观看时间、频道、时区和提醒优化</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>排入下一阶段页面优化</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>Tickets 页面</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-tickets/</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>未开始</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>待强化购票路径、城市/球队/日期关联入口</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>排入下一阶段页面优化</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>全站SEO技术项</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Sitemap / Schema / Canonical / 内链 / 图片alt</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>未开始</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>待统一审计</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>完成页面模块后统一执行</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>AdSense 技术准备项</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>全站验证 / ads.txt / 合规页面 / 广告加载开关</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>已加入开发清单，待上线前配置</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>已明确预留 head 验证、/ads.txt、Privacy Policy、About、Contact、Disclaimer、移动端体验和正式申请前检查项</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>网站内容完成并部署到 worldcup2026schedule.net 后，使用正式 AdSense 账号信息完成验证</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>AdSense 信任与合规页面</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>/privacy-policy/ /about/ /contact/ /disclaimer/</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>已创建4个合规基础页面；已加入footer入口和sitemap；每页包含独立说明、FAQ、canonical和Schema</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>上线前配置真实联系邮箱；拿到AdSense账号后再添加验证代码和ads.txt</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>AdSense 验证基础设施</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Head验证位 / AdSense脚本开关 / ads.txt / .env.example</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>已实现ADSENSE_PUBLISHER_ID、验证方式、脚本加载和ads.txt开关；默认构建不输出验证标签、不加载广告脚本、不写入假publisher ID</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>部署到worldcup2026schedule.net后，使用正式AdSense账号ID配置生产环境变量并验证源码</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Host Cities Phase B</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-schedule-host-cities/</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>已新增Region筛选、4个交互式城市比较卡、16个城市价值标签、16个Planning highlight模块；关键词密度回到4.67%</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>下一步可优化单个高优先级城市详情页，或继续做Groups页面工具化</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Host Cities Phase C</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>/world-cup-2026-schedule-host-cities/</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>已接入16张城市图片资源；新增8张视觉Featured City Cards，包含城市图、路线标签、球场、比赛数、容量和Open city guide入口</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>下一步可继续优化城市详情页，或为16个城市补充独立图片卡排序/横向滚动体验</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Host Cities 页面</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-host-cities/</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>已完成视觉城市卡补齐</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Featured City Cards 从8个扩展到16个，覆盖全部世界杯2026主办城市；已验证桌面/移动端无横向溢出、16张图片可加载。</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>下一步可做城市详情页深度优化或主办城市地图/路线规划模块。</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix host city planner navigation paths
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1052,6 +1052,43 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Host Cities 页面</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-host-cities/</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>已修复 Hero 城市规划器导航路径</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>修复 Show matching cities、Reset、Knockout hosts、Late tournament route 四个按钮；筛选后直接落到结果卡片区，URL 带 city/need 状态和 #host-city-results。</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>下一步可优化城市详情页内容和交互承接。</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Optimize host city detail pages
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1089,6 +1089,43 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Host City Detail Pages</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule/{city}/</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Completed deep optimization</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Upgraded all 16 city detail pages with city-specific H1/title/description, city image hero, schedule snapshot, match timeline, team chips, stage summary, stadium/travel/ticket planning cards, full fixture table and FAQ.</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>Next: second-pass schema and internal-link audit, or optimize Team Pages.</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Align groups page core keyword
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1126,6 +1126,43 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Groups ??</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-groups/</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>??????????</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>???????? world-cup-2026-schedule-groups???? URL?H1?Title?Description??????? /world-cup-2026-groups/ noindex ???</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>?????????????? Groups ??????????</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Optimize groups page keyword density
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1163,6 +1163,43 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Groups ??</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-groups/</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>??????????</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>?SEO????????1394????12?????48?????????????5?FAQ?????????3.95%???3%-5%???</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>???????Groups????/????????Team Pages?????</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Deepen groups page interaction
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1200,6 +1200,43 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Groups ??</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-groups/</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>??????????</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>??A-L?????URL?????12?group cards?72?fixture detail links?48?team chips?host city route links????????3.04%?????4.93%?</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>????????Team Pages????Groups?standings/bracket??????</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add groups qualification preview
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1237,6 +1237,43 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Groups ??</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-groups/</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>??? Phase C</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>????Qualification Path Panel?12???Standings Preview??????/???????????????3.92%??????????0?</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>??????Standings?????Groups???Live table???</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Make groups hero tool functional
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1274,6 +1274,43 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Groups ??</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-groups/</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>???Hero???????</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>???Quick facts??Group Finder????Group/Team?????Group Card?Standings?????Match Detail?Hero??????????????3.60%?</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>????????Hero??????????????????????????</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refine groups hero finder UX
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1311,6 +1311,43 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>Groups ??</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-groups/</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>???Hero Finder UX??</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>?Group/Team????????By group/By team???????Group A????A??????Team??????By team??????????3.58%?</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>??????????Hero????????Host Cities?Groups???????????</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Audit hero visual differentiation
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1348,6 +1348,43 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>??Hero??</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Schedule / PDF / Excel / Host Cities / Groups / Standings / Bracket / Dates / TV / Tickets</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>?????</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>??????Hero????????????Standings?Bracket?Dates?TV?Tickets?????Hero?Host Cities????????????</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>?????Phase Hero A.1?Standings hero redesign?</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Redesign standings hero and tables
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1385,6 +1385,43 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Standings ??</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-standings/</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>???Phase Hero A.1</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>????Hero???standings???Hero?Group Table Preview?12???????#group?????qualification status??????3.11%?</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>?????Standings Phase B????????????????????????</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add standings to primary navigation
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1422,6 +1422,43 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>??????</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>???Standings??</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>?????8???????????????Standings?Bracket????????????0?</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>???????Phase Hero A.2?Bracket hero redesign?</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Align standings keyword and URL
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1459,6 +1459,43 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>Standings ??</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule-standings/</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>?????????URL??</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>???????world-cup-2026-schedule-standings?URL???????/world-cup-2026-standings/??noindex????????????</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>???????Phase Hero A.2?Bracket hero redesign?</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add standings core keyword to headings
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="121">
   <si>
     <t>任务模块</t>
   </si>
@@ -387,6 +387,9 @@
   </si>
   <si>
     <t>下一步可做 Standings Phase B：表格筛选、状态解释和未来实时结果模型。</t>
+  </si>
+  <si>
+    <t>按要求将所有 H2、H3 加入核心关键词 World Cup 2026 Schedule Standings，并通过正文去重将关键词族密度控制在 3.52%。</t>
   </si>
 </sst>
 </file>
@@ -399,14 +402,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -862,148 +858,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1359,7 +1355,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="21.75" customWidth="1"/>
@@ -1486,7 +1482,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" ht="27" spans="1:7">
+    <row r="6" spans="1:7">
       <c r="A6" s="1" t="s">
         <v>27</v>
       </c>
@@ -1693,7 +1689,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" ht="27" spans="1:7">
+    <row r="15" spans="1:7">
       <c r="A15" s="1" t="s">
         <v>64</v>
       </c>
@@ -1716,7 +1712,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" ht="27" spans="1:7">
+    <row r="16" spans="1:7">
       <c r="A16" s="1" t="s">
         <v>67</v>
       </c>
@@ -1739,7 +1735,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" ht="27" spans="1:7">
+    <row r="17" spans="1:7">
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
@@ -1785,7 +1781,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" ht="40.5" spans="1:7">
+    <row r="19" ht="27" spans="1:7">
       <c r="A19" s="1" t="s">
         <v>76</v>
       </c>
@@ -1808,7 +1804,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" ht="27" spans="1:7">
+    <row r="20" spans="1:7">
       <c r="A20" s="1" t="s">
         <v>81</v>
       </c>
@@ -1854,7 +1850,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" ht="27" spans="1:7">
+    <row r="22" spans="1:7">
       <c r="A22" s="1" t="s">
         <v>81</v>
       </c>
@@ -1900,7 +1896,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" ht="27" spans="1:7">
+    <row r="24" spans="1:7">
       <c r="A24" s="1" t="s">
         <v>81</v>
       </c>
@@ -1969,7 +1965,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" ht="27" spans="1:7">
+    <row r="27" spans="1:7">
       <c r="A27" s="1" t="s">
         <v>104</v>
       </c>
@@ -2015,7 +2011,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" ht="27" spans="1:7">
+    <row r="29" spans="1:7">
       <c r="A29" s="1" t="s">
         <v>104</v>
       </c>
@@ -2058,6 +2054,29 @@
         <v>12</v>
       </c>
       <c r="G30" s="2">
+        <v>46166</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>117</v>
+      </c>
+      <c r="B31" t="s">
+        <v>114</v>
+      </c>
+      <c r="C31" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" t="s">
+        <v>120</v>
+      </c>
+      <c r="E31" t="s">
+        <v>119</v>
+      </c>
+      <c r="F31" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" s="2">
         <v>46166</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add schedule core keyword to headings
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="123">
   <si>
     <t>任务模块</t>
   </si>
@@ -390,6 +390,12 @@
   </si>
   <si>
     <t>按要求将所有 H2、H3 加入核心关键词 World Cup 2026 Schedule Standings，并通过正文去重将关键词族密度控制在 3.52%。</t>
+  </si>
+  <si>
+    <t>按要求将所有 H2、H3 加入核心关键词 World Cup 2026 Schedule；验证初始页、Date View、Team View、City View 可见标题均通过。</t>
+  </si>
+  <si>
+    <t>后续可继续做 Schedule 页结构化数据、性能与移动端表格体验复查。</t>
   </si>
 </sst>
 </file>
@@ -1355,7 +1361,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="21.75" customWidth="1"/>
@@ -2080,6 +2086,29 @@
         <v>46166</v>
       </c>
     </row>
+    <row r="32" spans="1:7">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" t="s">
+        <v>15</v>
+      </c>
+      <c r="C32" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" t="s">
+        <v>121</v>
+      </c>
+      <c r="E32" t="s">
+        <v>122</v>
+      </c>
+      <c r="F32" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" s="2">
+        <v>46166</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Add groups core keyword to headings
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="125">
   <si>
     <t>任务模块</t>
   </si>
@@ -396,6 +396,12 @@
   </si>
   <si>
     <t>后续可继续做 Schedule 页结构化数据、性能与移动端表格体验复查。</t>
+  </si>
+  <si>
+    <t>按要求将所有 H2、H3 加入核心关键词 World Cup 2026 Schedule Groups；关键词族密度 4.01%，保持在 3%-5%。</t>
+  </si>
+  <si>
+    <t>后续可继续做 Groups 页面视觉差异化和小组筛选体验复查。</t>
   </si>
 </sst>
 </file>
@@ -1361,7 +1367,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="21.75" customWidth="1"/>
@@ -2109,6 +2115,29 @@
         <v>46166</v>
       </c>
     </row>
+    <row r="33" spans="1:7">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>82</v>
+      </c>
+      <c r="C33" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" t="s">
+        <v>123</v>
+      </c>
+      <c r="E33" t="s">
+        <v>124</v>
+      </c>
+      <c r="F33" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="2">
+        <v>46166</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Add host cities core keyword to headings
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="127">
   <si>
     <t>任务模块</t>
   </si>
@@ -402,6 +402,12 @@
   </si>
   <si>
     <t>后续可继续做 Groups 页面视觉差异化和小组筛选体验复查。</t>
+  </si>
+  <si>
+    <t>按统一规则将所有 H2、H3 加入核心关键词 World Cup 2026 Schedule Host Cities；关键词族密度 4.48%，保持在 3%-5%。</t>
+  </si>
+  <si>
+    <t>后续可复查移动端长标题换行与城市卡片视觉密度。</t>
   </si>
 </sst>
 </file>
@@ -1367,11 +1373,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="21.75" customWidth="1"/>
-    <col min="2" max="2" width="39.375" customWidth="1"/>
+    <col min="2" max="2" width="41.5" customWidth="1"/>
     <col min="3" max="3" width="21.625" customWidth="1"/>
     <col min="4" max="4" width="141.375" customWidth="1"/>
     <col min="5" max="5" width="72.5" customWidth="1"/>
@@ -2138,6 +2144,29 @@
         <v>46166</v>
       </c>
     </row>
+    <row r="34" spans="1:7">
+      <c r="A34" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" t="s">
+        <v>125</v>
+      </c>
+      <c r="E34" t="s">
+        <v>126</v>
+      </c>
+      <c r="F34" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="2">
+        <v>46166</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Optimize PDF and Excel heading SEO
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="131">
   <si>
     <t>任务模块</t>
   </si>
@@ -408,6 +408,18 @@
   </si>
   <si>
     <t>后续可复查移动端长标题换行与城市卡片视觉密度。</t>
+  </si>
+  <si>
+    <t>PDF / Excel 页面</t>
+  </si>
+  <si>
+    <t>/world-cup-2026-schedule-pdf/ + /world-cup-2026-schedule-excel/</t>
+  </si>
+  <si>
+    <t>按统一规则完成两个下载页 H2/H3 核心关键词优化；PDF 使用 World Cup 2026 Schedule PDF，Excel 使用 World Cup 2026 Schedule Excel；补充实用说明以保持自然密度。</t>
+  </si>
+  <si>
+    <t>后续可继续做下载模块视觉密度、版本号提示和文件更新日期微文案。</t>
   </si>
 </sst>
 </file>
@@ -1373,13 +1385,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="21.75" customWidth="1"/>
-    <col min="2" max="2" width="41.5" customWidth="1"/>
+    <col min="2" max="2" width="70.375" customWidth="1"/>
     <col min="3" max="3" width="21.625" customWidth="1"/>
-    <col min="4" max="4" width="141.375" customWidth="1"/>
+    <col min="4" max="4" width="167.125" customWidth="1"/>
     <col min="5" max="5" width="72.5" customWidth="1"/>
     <col min="6" max="6" width="6.375" customWidth="1"/>
     <col min="7" max="7" width="10.625" customWidth="1"/>
@@ -2167,6 +2179,29 @@
         <v>46166</v>
       </c>
     </row>
+    <row r="35" spans="1:7">
+      <c r="A35" t="s">
+        <v>127</v>
+      </c>
+      <c r="B35" t="s">
+        <v>128</v>
+      </c>
+      <c r="C35" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" t="s">
+        <v>129</v>
+      </c>
+      <c r="E35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F35" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" s="2">
+        <v>46166</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Add download trust modules
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="134">
   <si>
     <t>任务模块</t>
   </si>
@@ -420,6 +420,15 @@
   </si>
   <si>
     <t>后续可继续做下载模块视觉密度、版本号提示和文件更新日期微文案。</t>
+  </si>
+  <si>
+    <t>Phase Download Trust A</t>
+  </si>
+  <si>
+    <t>完成 PDF / Excel 下载模块可信度与转化优化：增加任务推荐卡、更新时间、文件版本、体积、来源说明、独立站点说明、官方来源提醒和清晰下载按钮。</t>
+  </si>
+  <si>
+    <t>后续可继续做文件版本号自动化、下载点击事件统计和下载模块截图记录。</t>
   </si>
 </sst>
 </file>
@@ -1385,10 +1394,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="21.75" customWidth="1"/>
+    <col min="1" max="1" width="24.875" customWidth="1"/>
     <col min="2" max="2" width="70.375" customWidth="1"/>
     <col min="3" max="3" width="21.625" customWidth="1"/>
     <col min="4" max="4" width="167.125" customWidth="1"/>
@@ -1420,7 +1429,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="27" spans="1:7">
+    <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1627,7 +1636,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" ht="27" spans="1:7">
+    <row r="11" spans="1:7">
       <c r="A11" s="1" t="s">
         <v>47</v>
       </c>
@@ -1673,7 +1682,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" ht="27" spans="1:7">
+    <row r="13" spans="1:7">
       <c r="A13" s="1" t="s">
         <v>56</v>
       </c>
@@ -1972,7 +1981,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" ht="40.5" spans="1:7">
+    <row r="26" ht="27" spans="1:7">
       <c r="A26" s="1" t="s">
         <v>99</v>
       </c>
@@ -2199,6 +2208,29 @@
         <v>12</v>
       </c>
       <c r="G35" s="2">
+        <v>46166</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" t="s">
+        <v>131</v>
+      </c>
+      <c r="B36" t="s">
+        <v>128</v>
+      </c>
+      <c r="C36" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" t="s">
+        <v>132</v>
+      </c>
+      <c r="E36" t="s">
+        <v>133</v>
+      </c>
+      <c r="F36" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="2">
         <v>46166</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add trust page prelaunch checklist
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="138">
   <si>
     <t>任务模块</t>
   </si>
@@ -429,6 +429,18 @@
   </si>
   <si>
     <t>后续可继续做文件版本号自动化、下载点击事件统计和下载模块截图记录。</t>
+  </si>
+  <si>
+    <t>Trust Pages Pre-Launch Architecture</t>
+  </si>
+  <si>
+    <t>/about/ + /contact/ + /privacy-policy/ + /disclaimer/</t>
+  </si>
+  <si>
+    <t>已建立信任页面上线前信息采集清单；记录 owner/operator、联系邮箱、隐私工具、AdSense、ads.txt、免责声明等缺失信息；明确 AdSense 提交前阻塞项，避免编造主体信息。</t>
+  </si>
+  <si>
+    <t>上线前需要用户补充真实主体信息、确认联系邮箱可用、确认隐私与广告配置后再提交 AdSense。</t>
   </si>
 </sst>
 </file>
@@ -1394,14 +1406,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="24.875" customWidth="1"/>
+    <col min="1" max="1" width="39.375" customWidth="1"/>
     <col min="2" max="2" width="70.375" customWidth="1"/>
     <col min="3" max="3" width="21.625" customWidth="1"/>
-    <col min="4" max="4" width="167.125" customWidth="1"/>
-    <col min="5" max="5" width="72.5" customWidth="1"/>
+    <col min="4" max="4" width="167.625" customWidth="1"/>
+    <col min="5" max="5" width="90.625" customWidth="1"/>
     <col min="6" max="6" width="6.375" customWidth="1"/>
     <col min="7" max="7" width="10.625" customWidth="1"/>
   </cols>
@@ -2234,6 +2246,29 @@
         <v>46166</v>
       </c>
     </row>
+    <row r="37" spans="1:7">
+      <c r="A37" t="s">
+        <v>134</v>
+      </c>
+      <c r="B37" t="s">
+        <v>135</v>
+      </c>
+      <c r="C37" t="s">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s">
+        <v>136</v>
+      </c>
+      <c r="E37" t="s">
+        <v>137</v>
+      </c>
+      <c r="F37" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="2">
+        <v>46167</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Add launch readiness technical audit
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="142">
   <si>
     <t>任务模块</t>
   </si>
@@ -441,6 +441,18 @@
   </si>
   <si>
     <t>上线前需要用户补充真实主体信息、确认联系邮箱可用、确认隐私与广告配置后再提交 AdSense。</t>
+  </si>
+  <si>
+    <t>Phase Launch Readiness A</t>
+  </si>
+  <si>
+    <t>全站上线前技术体检</t>
+  </si>
+  <si>
+    <t>完成上线前技术体检清单：检查 sitemap、robots.txt、ads.txt、canonical、noindex、footer 信任入口、AdSense 默认安全状态、关键页面移动端溢出和 H1 数量。</t>
+  </si>
+  <si>
+    <t>上线前需补齐 static 404.html；继续完成 trust-pages-prelaunch-info-checklist.md 中真实主体、联系邮箱、隐私和 AdSense 信息。</t>
   </si>
 </sst>
 </file>
@@ -1406,14 +1418,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="39.375" customWidth="1"/>
     <col min="2" max="2" width="70.375" customWidth="1"/>
     <col min="3" max="3" width="21.625" customWidth="1"/>
     <col min="4" max="4" width="167.625" customWidth="1"/>
-    <col min="5" max="5" width="90.625" customWidth="1"/>
+    <col min="5" max="5" width="132.125" customWidth="1"/>
     <col min="6" max="6" width="6.375" customWidth="1"/>
     <col min="7" max="7" width="10.625" customWidth="1"/>
   </cols>
@@ -1717,7 +1729,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" ht="27" spans="1:7">
+    <row r="14" spans="1:7">
       <c r="A14" s="1" t="s">
         <v>60</v>
       </c>
@@ -2266,6 +2278,29 @@
         <v>12</v>
       </c>
       <c r="G37" s="2">
+        <v>46167</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" t="s">
+        <v>138</v>
+      </c>
+      <c r="B38" t="s">
+        <v>139</v>
+      </c>
+      <c r="C38" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" t="s">
+        <v>140</v>
+      </c>
+      <c r="E38" t="s">
+        <v>141</v>
+      </c>
+      <c r="F38" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="2">
         <v>46167</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add static 404 page
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="146">
   <si>
     <t>任务模块</t>
   </si>
@@ -453,6 +453,18 @@
   </si>
   <si>
     <t>上线前需补齐 static 404.html；继续完成 trust-pages-prelaunch-info-checklist.md 中真实主体、联系邮箱、隐私和 AdSense 信息。</t>
+  </si>
+  <si>
+    <t>Phase Launch Readiness B</t>
+  </si>
+  <si>
+    <t>Static 404 Page and Error-State UX</t>
+  </si>
+  <si>
+    <t>创建静态 404.html；未知 URL 在最新预览服务中返回 HTTP 404 并显示 Page Not Found；页面 noindex，不进 sitemap，保留 Schedule/PDF/Excel/Host Cities/Contact 和信任页入口。</t>
+  </si>
+  <si>
+    <t>上线部署后需测试真实生产未知 URL 是否返回 404，并确认托管平台使用 /404.html。</t>
   </si>
 </sst>
 </file>
@@ -1418,13 +1430,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="39.375" customWidth="1"/>
     <col min="2" max="2" width="70.375" customWidth="1"/>
     <col min="3" max="3" width="21.625" customWidth="1"/>
-    <col min="4" max="4" width="167.625" customWidth="1"/>
+    <col min="4" max="4" width="181" customWidth="1"/>
     <col min="5" max="5" width="132.125" customWidth="1"/>
     <col min="6" max="6" width="6.375" customWidth="1"/>
     <col min="7" max="7" width="10.625" customWidth="1"/>
@@ -2304,6 +2316,29 @@
         <v>46167</v>
       </c>
     </row>
+    <row r="39" spans="1:7">
+      <c r="A39" t="s">
+        <v>142</v>
+      </c>
+      <c r="B39" t="s">
+        <v>143</v>
+      </c>
+      <c r="C39" t="s">
+        <v>9</v>
+      </c>
+      <c r="D39" t="s">
+        <v>144</v>
+      </c>
+      <c r="E39" t="s">
+        <v>145</v>
+      </c>
+      <c r="F39" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="2">
+        <v>46167</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Add production deployment checklist
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="150">
   <si>
     <t>任务模块</t>
   </si>
@@ -465,6 +465,18 @@
   </si>
   <si>
     <t>上线部署后需测试真实生产未知 URL 是否返回 404，并确认托管平台使用 /404.html。</t>
+  </si>
+  <si>
+    <t>Phase Launch Readiness C</t>
+  </si>
+  <si>
+    <t>Production Deployment Checklist</t>
+  </si>
+  <si>
+    <t>完成生产部署清单：明确 worldcup2026schedule.net 部署前配置、环境变量、DNS/HTTPS、sitemap/robots/ads.txt、404、下载文件、Search Console 和 AdSense 验证步骤。</t>
+  </si>
+  <si>
+    <t>后续需要选择托管平台、配置 DNS/HTTPS、启用联系邮箱，并在生产环境验证 sitemap、robots、ads.txt、404 和核心页面。</t>
   </si>
 </sst>
 </file>
@@ -1430,7 +1442,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="39.375" customWidth="1"/>
@@ -2339,6 +2351,29 @@
         <v>46167</v>
       </c>
     </row>
+    <row r="40" spans="1:7">
+      <c r="A40" t="s">
+        <v>146</v>
+      </c>
+      <c r="B40" t="s">
+        <v>147</v>
+      </c>
+      <c r="C40" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" t="s">
+        <v>148</v>
+      </c>
+      <c r="E40" t="s">
+        <v>149</v>
+      </c>
+      <c r="F40" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" s="2">
+        <v>46167</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Make schedule page the homepage
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2542,6 +2542,43 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>Homepage Routing</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>/ -&gt; /world-cup-2026-schedule/</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>Retired the thin standalone root homepage. Root now redirects to the World Cup 2026 Schedule page, Home and logo navigation point to the schedule page, sitemap excludes root, and Cloudflare _redirects includes a 301 rule.</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>Continue with Team Page Content System Redesign and support-page optimization based on the low-quality audit.</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add team directory and SEO framework
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2579,6 +2579,43 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>Team Pages Entry + SEO Framework</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-schedule/ and 48 team pages</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>Added a visible Team Schedule Directory on the homepage schedule hub with 48 unique team page links. Added Teams navigation anchor. Created team-pages SEO keyword framework with core keyword rule, long-tail keyword families, metadata structure, H1/H2/H3 structure and per-team content angles.</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>Next: optimize team pages one by one, starting with Mexico, United States and Canada, using unique route-specific copy and avoiding bulk template content.</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebuild team schedule pages
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2616,6 +2616,43 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>Team Pages Rebuild</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>48 Team schedule pages</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>Completed first reconstruction</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>Rebuilt the 48 Team pages from thin template pages into team-route pages with unique group, opponent, city, stadium and match-detail data. Added team fixture cards, group opponent context, host-city route, usage cards, related planning links and FAQ. Team pages now have 1087-1154 visible words and 3.49%-4.22% weighted core keyword density.</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>Next: manually enrich high-search team pages first: Mexico, United States, Canada, Argentina, Brazil, England, France, Germany, Spain and Portugal.</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebuild dates support page
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2653,6 +2653,43 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Phase Support Pages A.1</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-dates/</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>Rebuilt the World Cup 2026 Dates page into a timeline planner with stage table, key-date cards, travel/download decision paths, source notes, visual schedule image and HowTo schema. Updated Title, Description, H1, H2/H3 structure and SEO reference files. Visible word count is 1401 and weighted keyword density is 4.85%.</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Next: Phase Support Pages A.2 - rebuild /world-cup-2026-tv-schedule/.</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebuild TV schedule support page
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2690,6 +2690,43 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>Phase Support Pages A.2</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-tv-schedule/</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>Rebuilt the World Cup 2026 TV Schedule page into a viewing planner with TV-specific hero, broadcaster verification paths, match-time workflow, key match-window cards, country viewing checks, source notes and HowTo schema. Visible word count is 1796 and weighted keyword density is 4.45%.</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>Next: rebuild /where-to-watch-world-cup-2026/ or continue support-page remediation for Bracket, Final and Tickets before launch.</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Enhance South Korea team page experience
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2727,6 +2727,43 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>Team Page Deep Optimization</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-teams/south-korea-schedule/</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>Updated the South Korea page experience without changing core keyword, Title, Description, H1, H2 or H3. Added team snapshot, Group A mini standings, group fixtures, qualification route panel, role-based lineup board, route city cards and TV guide link. Visible word count is 1568 and weighted keyword density is 3.06%.</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>Next: use this Korea page pattern to optimize Mexico, United States or another high-priority team page one by one.</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Redesign South Korea team hero
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1,19 +1,35 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务进度" sheetId="1" state="visible" r:id="rId1"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
+  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">openpyxl</dc:creator>
+  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-05-24T04:00:00Z</dcterms:created>
+  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-05-25T03:54:34Z</dcterms:modified>
+  <cp:lastModifiedBy>Tony</cp:lastModifiedBy>
+</cp:coreProperties>
+</file>
+
+<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties">
+  <property name="ICV" fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2">
+    <vt:lpwstr xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">6BD6F9F82A214158A4D5BCACF26D605C_12</vt:lpwstr>
+  </property>
+  <property name="KSOProductBuildVer" fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3">
+    <vt:lpwstr xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">2052-12.1.0.26375</vt:lpwstr>
+  </property>
+  <property name="CalculationRule" fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4">
+    <vt:i4 xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">0</vt:i4>
+  </property>
+</Properties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="20">
@@ -747,7 +763,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1029,13 +1045,27 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务进度" sheetId="1" state="visible" r:id="rId1"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2764,6 +2794,43 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>South Korea Team Hero Redesign</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-teams/south-korea-schedule/</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>Changed the South Korea page top from the generic stadium hero to a MatchTimes-style team profile card with flag, Korea Republic display name, preserved H1, favorite control, coach/squad/upcoming match stats and quick route anchors. Title, Description, H1, H2 and H3 stayed unchanged. Visible word count is 1549 and weighted keyword density is 3.10%.</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>Next: use this profile-card pattern to rebuild priority Team pages one by one, starting with Mexico, United States, Canada, Argentina, Brazil and England.</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roll out team profile experience
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2831,6 +2831,43 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>All Team Pages Profile Interaction Rollout</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>48 Team schedule pages</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>Generalized the South Korea profile-card interaction pattern across all 48 Team pages. Each page now has a team profile hero, flag, display name, coach/squad/upcoming-match cards, favorite control, group overview anchors, qualification path, role-based lineup board, route city cards and TV guide link using that team-specific schedule data.</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>Next: deep optimize high-search Team pages one by one, starting with Mexico, United States, Canada, Brazil, Argentina and England. Do not treat this rollout as a substitute for editorial page-by-page enrichment.</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roll out match detail SEO keyword framework
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2868,6 +2868,43 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>Match Detail Pages SEO Keyword Rollout</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>104 match detail pages</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>Applied the core keyword pattern {Home} vs {Away} World Cup 2026 schedule to all match detail pages. Updated Title, Description, H1, H2/H3 variants, Article schema descriptions and FAQ wording. Batch validation found 0 pages outside checks, longest title 59 characters, longest description 145 characters and keyword density range 3.35%-4.47%.</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>Next: manually enrich priority match pages around high-search teams and opening matches while preserving the current core keyword framework.</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add retention paths to early match pages
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2905,6 +2905,43 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>Phase Match Detail UX A.1</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>Match detail pages 1-12</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>Added an Early match planner retention module to Match 1-12 with shortcuts for kickoff/timezone, group route, team pages, host city guide, next connected match, PDF and Excel downloads. Batch validation confirmed the module appears only on Match 1-12, not after Match 12, with keyword density range 3.36%-4.47%.</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>Next: selectively apply deeper match UX to high-demand matches or opening-week team routes after reviewing search priority.</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Polish opening match detail page
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2942,6 +2942,43 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>Phase Match Detail UX A.2</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>/world-cup-2026-match/1-mexico-vs-south-africa/</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>Added a Match 1-only Opening match hub with first-kickoff badge, opener context, practical confirmation cards, Group A follow-up cards and direct links to Mexico, South Africa, Group A, Mexico City and Match 2. Validation confirmed 104 match pages checked, 0 pages outside checks, keyword density range 3.12%-4.07%, and the opening module appears only on Match 1.</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>Next: apply page-specific deep polish to other high-demand match pages such as United States, Mexico, Canada, knockout fixtures and the final without turning them into one template.</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Optimize USA match detail pages
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -2979,6 +2979,43 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>Phase Match Detail UX A.3</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>USA match detail pages: Match 4, 29, 57</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>Added a United States route planner module only to the three USA match detail pages. Each page now connects the match query to USA route context, opponent context, Group D, standings, city guide, TV guide and the full United States three-match route. Batch validation checked 104 match pages with 0 SEO failures; USA page keyword densities are 3.85%, 3.86% and 3.83%.</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>Next: continue selective deep polish for Mexico route pages, Canada route pages, final and semifinals instead of bulk editing every match page.</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Optimize Mexico match detail pages
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -3016,6 +3016,43 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>Phase Match Detail UX A.4</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>Mexico match detail pages: Match 1, 28, 55</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>Added a Mexico route planner module only to the three Mexico match detail pages. Each page now connects the match query to Mexico route context, Mexico City or Guadalajara, opponent context, Group A, standings, TV guide and ticket guide. Batch validation checked 104 match pages with 0 SEO failures; Mexico page keyword densities are 4.04%, 3.78% and 3.34%.</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>Next: continue host-nation clustering with Canada route pages, then optimize final and semifinal match pages.</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Optimize Canada match detail pages
</commit_message>
<xml_diff>
--- a/task-progress/wc2026schedule-task-progress.xlsx
+++ b/task-progress/wc2026schedule-task-progress.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="39.375" customWidth="1" min="1" max="1"/>
@@ -3053,6 +3053,43 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>Phase Match Detail UX A.5</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>Canada match detail pages: Match 3, 27, 49</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>Added a Canada route planner module only to the three Canada match detail pages. Each page now connects the match query to Canada route context, Toronto or Vancouver, opponent context, Group B, standings, TV guide and ticket guide. Batch validation checked 104 match pages with 0 SEO failures; Canada page keyword densities are 4.22%, 3.37% and 3.36%.</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>Next: host-nation route clusters are complete. Optimize final, semifinals and third-place match pages as event pages.</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>